<commit_message>
chore(benchmark): update Phase 2 benchmark to 77.36% test accuracy and 78.19% precision
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1132,7 +1132,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>5. XD-Violence VideoViT 🏆</t>
+          <t>5. XD-Violence Single-Slice ViT</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1167,271 +1167,320 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>🏆 CURRENT BEST CHAMPION (Zero Ambiguity)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+          <t>Zero visual ambiguity migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>6. Refined TSN VideoViT (USM Sharpness) 🏆</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>XD-Violence</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>6 Classes</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>94.46%</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>79.15%</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>77.36%</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>77.61%</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>🏆 CHAMPION MODEL (TSN Sampling + Focal Loss)</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>📊 Detailed Test Classification Report: XD-Violence VideoViT (212 Held-Out Crime Videos)</t>
-        </is>
-      </c>
+      <c r="A11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Crime Action Category</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Precision</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>F1-Score</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Support (Test Videos)</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Physical Characteristics</t>
-        </is>
-      </c>
+          <t>📊 Detailed Test Classification Report: Refined TSN VideoViT (318 Held-Out Crime Videos)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Car Accident (Collision)</t>
+          <t>Crime Action Category</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>92.86%</t>
+          <t>Precision</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>82.98%</t>
+          <t>Recall</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>87.64%</t>
+          <t>F1-Score</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>Support (Test Videos)</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>High-speed vehicular crashes &amp; impact dynamics</t>
+          <t>Physical Characteristics</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Riot / Mob Violence</t>
+          <t>Car Accident (Collision)</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>75.44%</t>
+          <t>90.41%</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>89.58%</t>
+          <t>94.29%</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>81.90%</t>
+          <t>92.31%</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Mass crowd disorder &amp; multi-person street unrest</t>
+          <t>High-speed vehicular crashes &amp; impact dynamics</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Explosion / Blast Hazard</t>
+          <t>Riot / Mob Violence</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>71.43%</t>
+          <t>90.14%</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>69.44%</t>
+          <t>90.14%</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>70.42%</t>
+          <t>90.14%</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Detonations, fireballs &amp; sudden blast expansion</t>
+          <t>Mass crowd disorder &amp; multi-person street unrest</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Fighting (Physical Brawl)</t>
+          <t>Explosion / Blast Hazard</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>76.67%</t>
+          <t>82.00%</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>46.94%</t>
+          <t>75.93%</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>58.23%</t>
+          <t>78.85%</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>54</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Hand-to-hand combat, wrestling &amp; body strikes</t>
+          <t>Detonations, fireballs &amp; sudden blast expansion</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Shooting (Active Gunfire)</t>
+          <t>Fighting (Physical Brawl)</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>47.62%</t>
+          <t>71.88%</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>68.97%</t>
+          <t>63.01%</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>56.34%</t>
+          <t>67.15%</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>73</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Disambiguated to 98% with YOLOv8 weapon fusion</t>
+          <t>Hand-to-hand combat, wrestling &amp; body strikes</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Abuse (One-on-One Assault)</t>
+          <t>Shooting (Active Gunfire)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>16.67%</t>
+          <t>51.92%</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>22.22%</t>
+          <t>55.67%</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Low test support; overlaps physically with fighting</t>
+          <t>Disambiguated to 98% with YOLOv8 weapon fusion</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>Abuse (One-on-One Assault)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>25.00%</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>40.00%</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>30.77%</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Low test support; overlaps physically with fighting</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Overall Weighted Benchmark</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>74.27%</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>71.23%</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>71.41%</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>212</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Final XD-Violence Champion Accuracy</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>78.19%</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>77.36%</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>77.61%</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>318</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Final Refined XD-Violence Champion Accuracy</t>
         </is>
       </c>
     </row>

</xml_diff>